<commit_message>
Add merdiven, tank isim plakası; update çatı iskeleti with image 5 data
- Added Tank İsim Plakası (TI-1~TI-4, S275J2+304SS, 5.18 kg) to
  Manhol+Temizleme sheet as new section
- Added Merdiven+Korkuluk (23 structural items + fasteners, 1777.0 kg)
  to Manhol+Temizleme sheet based on MKD-210 drawing
- Rewrote Konik Çatı İskeleti sheet with complete image 5 breakdown:
  CK1×12, CK2×12, CK3×24, CK4×24, KL1×1, W1×24, W2×1, YC1×12, YC2×12
  Fixed P1 rafter weight: 155.5 kg (was 188.8); corrected KL1 P9/P11/P12
- Updated Toplam Ağırlık Özeti: çatı = 5454.0 kg, merdiven = 1777.0 kg,
  added İsim Plakası row

https://claude.ai/code/session_017Cpp1ZZqefHw5fPaaS3WRF
</commit_message>
<xml_diff>
--- a/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
+++ b/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
@@ -5861,7 +5861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7573,15 +7573,1137 @@
       </c>
       <c r="G62" s="9" t="inlineStr"/>
     </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>TANK İSİM PLAKASI  (1 Adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>ADET</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+AĞIRLIK(kg)</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM
+AĞIRLIK(kg)</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM TÜRÜ</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 215×6 ......... 230</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 230×6 ......... 230</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B68" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 25×6 ......... 230</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B69" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>BOLT/NVT NO.5-40 UNC</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>304 S.S</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>TOPLAM AĞIRLIK: 5.18 Kg</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="G70" s="9" t="inlineStr"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>MERDİVEN + KORKULUK  (1 Komple)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>ADET</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+AĞIRLIK(kg)</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM
+AĞIRLIK(kg)</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM TÜRÜ</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B74" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 7550.5</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 972.5</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 6190</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B77" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 899.5</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B78" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 8057.5</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B79" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 1069.5</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 6603.5</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B81" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 1002.5</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B82" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 1079</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F82" s="4" t="n">
+        <v>248.4</v>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 ......... 750</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B84" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>NPU100 ......... 1080</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F84" s="4" t="n">
+        <v>138</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B85" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>NPU100 ......... 1178.5</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B86" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 8×100 ......... 260</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>S355J2</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F86" s="4" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B87" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 325.5</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>14A</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 325.5</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F88" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×70 ......... 180</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B90" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 899.5</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F90" s="4" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B91" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 630</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B92" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 1002.5</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F92" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B93" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 1238</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B94" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>L60×6 ......... 1020</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F94" s="4" t="n">
+        <v>140.4</v>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B95" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>HANDRAİL (1 1/4" STD.SCH PIPE) 70000</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="F95" s="6" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Bükme</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B96" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 5×50 ......... 70000</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="F96" s="4" t="n">
+        <v>137.5</v>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B97" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 5×150 ......... 34000</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t>Kesim</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="n"/>
+      <c r="B98" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>M10×30  BOLT</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>A193 GR B7</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n"/>
+      <c r="B99" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>M10  NUT</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>A194 GR 2H</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="n"/>
+      <c r="B100" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>M10  WASHER</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>A194 GR 2H</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n"/>
+      <c r="B101" s="6" t="n">
+        <v>136</v>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>M12×40  BOLT</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>A193 GR B7</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n"/>
+      <c r="B102" s="4" t="n">
+        <v>136</v>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>M12  NUT</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>A194 GR 2H</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="n"/>
+      <c r="B103" s="6" t="n">
+        <v>136</v>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>M12  WASHER</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>A194 GR 2H</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F103" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G103" s="6" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>TOPLAM AĞIRLIK: 1777.0 Kg</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="n">
+        <v>1777</v>
+      </c>
+      <c r="G104" s="9" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="11">
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A104:E104"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A72:G72"/>
+    <mergeCell ref="A64:G64"/>
     <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A70:E70"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7593,30 +8715,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KONİK ÇATI YAPISAL İSKELET MALZEME LİSTESİ  (Çizim: KEY199MECEQP2004)</t>
+          <t>KONİK ÇATI YAPISAL İSKELET MALZEME LİSTESİ  (TOPLAM: 5454.0 kg)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>CK1 MONTAJ GRUBU  (12 Adet)  —  Rafterlar UNP240</t>
+          <t>CK1  —  UNP240 Rafter  (12 çatım adedi)</t>
         </is>
       </c>
     </row>
@@ -7629,12 +8752,12 @@
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>ADET
-(1 grp)</t>
+(1 asm)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AÇIKLAMA</t>
+          <t>PROFİL / AÇIKLAMA</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -7651,16 +8774,22 @@
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>BİRİM
-AĞIRLIK(kg)</t>
+Kg</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>TOPLAM AĞIRLIK
-(tüm grp) kg</t>
+          <t>1 ASM
+TOPLAM kg</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>×12
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>İŞLEM</t>
         </is>
@@ -7689,12 +8818,15 @@
         <v>5685</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>188.8</v>
+        <v>155.5</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2265.6</v>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+        <v>155.5</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>1866</v>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7711,7 +8843,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>PL10×113  PLAKA</t>
+          <t>PL10×113  Plaka</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -7726,9 +8858,12 @@
         <v>1.8</v>
       </c>
       <c r="G5" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H5" s="6" t="n">
         <v>43.2</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7745,7 +8880,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>PL10×98   PLAKA</t>
+          <t>PL10×95   Plaka</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -7754,15 +8889,18 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>182</v>
+        <v>152</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+        <v>2.5</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7779,7 +8917,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>PL10×221  PLAKA</t>
+          <t>PL10×221  Plaka</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -7794,9 +8932,12 @@
         <v>2.7</v>
       </c>
       <c r="G7" s="6" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>32.4</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7813,7 +8954,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>PL10×162  PLAKA</t>
+          <t>PL10×162  Plaka</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -7828,9 +8969,12 @@
         <v>1.9</v>
       </c>
       <c r="G8" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>22.8</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7839,18 +8983,18 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>ALT TOPLAM:</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>2397.6</v>
-      </c>
-      <c r="H9" s="9" t="inlineStr"/>
+          <t>ALT TOPLAM  (×12):</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>1994.4</v>
+      </c>
+      <c r="I9" s="9" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>CK2 MONTAJ GRUBU  (12 Adet)  —  Rafterlar UNP240</t>
+          <t>CK2  —  UNP240 Rafter  (12 çatım adedi)</t>
         </is>
       </c>
     </row>
@@ -7863,12 +9007,12 @@
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>ADET
-(1 grp)</t>
+(1 asm)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>AÇIKLAMA</t>
+          <t>PROFİL / AÇIKLAMA</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -7885,16 +9029,22 @@
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>BİRİM
-AĞIRLIK(kg)</t>
+Kg</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>TOPLAM AĞIRLIK
-(tüm grp) kg</t>
+          <t>1 ASM
+TOPLAM kg</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>×12
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>İŞLEM</t>
         </is>
@@ -7923,12 +9073,15 @@
         <v>5685</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>188.8</v>
+        <v>155.5</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>2265.6</v>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+        <v>155.5</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>1866</v>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7945,7 +9098,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>PL10×113  PLAKA</t>
+          <t>PL10×113  Plaka</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -7960,9 +9113,12 @@
         <v>1.8</v>
       </c>
       <c r="G14" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H14" s="6" t="n">
         <v>43.2</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -7979,7 +9135,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>PL10×98   PLAKA</t>
+          <t>PL10×95   Plaka</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -7988,15 +9144,18 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>182</v>
+        <v>152</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+        <v>2.5</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -8013,7 +9172,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>PL10×189  PLAKA</t>
+          <t>PL10×189  Plaka</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -8025,12 +9184,15 @@
         <v>232</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
+        <v>2.5</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -8047,7 +9209,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>PL10×139  PLAKA</t>
+          <t>PL10×139  Plaka</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -8062,9 +9224,12 @@
         <v>2</v>
       </c>
       <c r="G17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
@@ -8073,18 +9238,18 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>ALT TOPLAM:</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="n">
-        <v>2400</v>
-      </c>
-      <c r="H18" s="9" t="inlineStr"/>
+          <t>ALT TOPLAM  (×12):</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>1993.2</v>
+      </c>
+      <c r="I18" s="9" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>KL1 MONTAJ GRUBU  (1 Adet)  —  Merkezi Kolon PIP 323.9×8</t>
+          <t>CK3  —  UNP200 Purlin  (24 adet)</t>
         </is>
       </c>
     </row>
@@ -8097,12 +9262,12 @@
       <c r="B21" s="2" t="inlineStr">
         <is>
           <t>ADET
-(1 grp)</t>
+(1 asm)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>AÇIKLAMA</t>
+          <t>PROFİL / AÇIKLAMA</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -8119,16 +9284,22 @@
       <c r="F21" s="2" t="inlineStr">
         <is>
           <t>BİRİM
-AĞIRLIK(kg)</t>
+Kg</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>TOPLAM AĞIRLIK
-(tüm grp) kg</t>
+          <t>1 ASM
+TOPLAM kg</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>×24
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>İŞLEM</t>
         </is>
@@ -8137,7 +9308,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
@@ -8145,7 +9316,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>PIP 323.9×8  BORU</t>
+          <t>UNP200</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -8154,672 +9325,1112 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>9369</v>
+        <v>1227</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>580.2</v>
+        <v>31</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>580.2</v>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+        <v>31</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>744</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>PL25×1800  PLAKA</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>497.3</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>497.3</v>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>PL15×250  PLAKA</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>4618</v>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>137.1</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>137.1</v>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>ALT TOPLAM:</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>1214.6</v>
-      </c>
-      <c r="H25" s="9" t="inlineStr"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>DİĞER YAPISAL ELEMANLAR  (Toplam plan miktarları)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="35" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×24):</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>744</v>
+      </c>
+      <c r="I23" s="9" t="inlineStr"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>CK4  —  UNP200 Purlin  (24 adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>POZ</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>ADET
-(TOPLAM)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>AÇIKLAMA</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
+(1 asm)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>MALZEME</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>BOY
 (mm)</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>BİRİM
-AĞIRLIK(kg)</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>TOPLAM
-AĞIRLIK(kg)</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+Kg</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>1 ASM
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>×24
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>İŞLEM</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>UNP200</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>677</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>410.4</v>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×24):</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>410.4</v>
+      </c>
+      <c r="I28" s="9" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>KL1  —  Merkezi Kolon PIP 323.9×8  (1 adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="35" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ADET
+(1 asm)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>BOY
+(mm)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+Kg</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>1 ASM
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>×1
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>PIP 323.9×8  Boru</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>9369</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>580.2</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>580.2</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>580.2</v>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>PL25×1800  Plaka</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>497.3</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>497.3</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>497.3</v>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>PL15×250   Plaka</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>4618</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>137.1</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>137.1</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>137.1</v>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>PL10×200   Plaka</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>5341</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>PL25×750   Plaka</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>750</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>PL10×150   Plaka</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>PL10×513   Plaka</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>PL20×600   Plaka</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×1):</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>1507.2</v>
+      </c>
+      <c r="I40" s="9" t="inlineStr"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>W1  —  Ayak Gusset Grubu  (24 adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="35" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>ADET
+(1 asm)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>BOY
+(mm)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+Kg</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>1 ASM
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>×24
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>PL10×300  PLAKA</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="B44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>PL10×300  Plaka</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>S235JR</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E44" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="F29" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G29" s="4" t="n">
+      <c r="F44" s="4" t="n">
         <v>7.1</v>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="G44" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>170.4</v>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>PL10×200  Plaka</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>PL10×200  Plaka</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>PL10×248  Plaka</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>299</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Kesim+Kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×24):</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>403.2</v>
+      </c>
+      <c r="I48" s="9" t="inlineStr"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>W2  —  Üst Halka Plakası  (1 adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="35" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>ADET
+(1 asm)</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>BOY
+(mm)</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+Kg</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>1 ASM
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>×1
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>PL15×750  PLAKA</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="B52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>PL15×750  Plaka</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>S235JR</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n">
+      <c r="E52" s="4" t="n">
         <v>750</v>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="F52" s="4" t="n">
         <v>51.6</v>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="G52" s="4" t="n">
         <v>51.6</v>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H52" s="4" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>UNP200</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>PL15×100  Plaka</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>S235JR</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n">
-        <v>1227</v>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>744</v>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="E53" s="6" t="n">
+        <v>1916</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="G53" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="H53" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>UNP200</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×1):</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="I54" s="9" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>YC1  —  Yatay Çelik 1  (12 adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="35" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ADET
+(1 asm)</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>BOY
+(mm)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+Kg</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>1 ASM
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>×12
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>L60×5  Köşebent</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>S235JR</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n">
-        <v>677</v>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>410.4</v>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="E58" s="4" t="n">
+        <v>1931</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>187.2</v>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>L80×8  KÖŞEBENTİ</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×12):</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>187.2</v>
+      </c>
+      <c r="I59" s="9" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>YC2  —  Yatay Çelik 2  (12 adet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="35" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ADET
+(1 asm)</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>BOY
+(mm)</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+Kg</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>1 ASM
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>×12
+TOPLAM kg</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>İŞLEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>L60×5  Köşebent</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>S235JR</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n">
-        <v>1931</v>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>223.2</v>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="E63" s="4" t="n">
+        <v>1954</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>230.4</v>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
         <is>
           <t>Kesim+Kaynak</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>L80×8  KÖŞEBENTİ</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>1984</v>
-      </c>
-      <c r="F34" s="6" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="G34" s="6" t="n">
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>ALT TOPLAM  (×12):</t>
+        </is>
+      </c>
+      <c r="H64" s="9" t="n">
         <v>230.4</v>
       </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>PL10×200  PLAKA</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>5341</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>84.2</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>84.2</v>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>PL25×750  PLAKA</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>750</v>
-      </c>
-      <c r="F36" s="6" t="n">
-        <v>86</v>
-      </c>
-      <c r="G36" s="6" t="n">
-        <v>86</v>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>PL10×200  PLAKA</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="F37" s="4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G37" s="4" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>Kesim</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>P14</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>PL10×200  PLAKA</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F38" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G38" s="6" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>Kesim</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>P15</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>PL10×248  PLAKA</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>299</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>Kesim</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>P16</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>PL10×150  PLAKA</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>250</v>
-      </c>
-      <c r="F40" s="6" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G40" s="6" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>Kesim</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>P17</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>PL10×513  PLAKA</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>675</v>
-      </c>
-      <c r="F41" s="4" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>P18</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>PL20×600  PLAKA</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>600</v>
-      </c>
-      <c r="F42" s="6" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="G42" s="6" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>Kesim+Kaynak</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>P19</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>PL15×100  PLAKA</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>1916</v>
-      </c>
-      <c r="F43" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="G43" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>Kesim</t>
+      <c r="I64" s="9" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>NOT: Çizimden alınan TOPLAM AĞIRLIK = 5454.0 Kg  (1 komple çatı iskeleti için verilmiştir).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A25:F25"/>
+  <mergeCells count="20">
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A66:I66"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A42:I42"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A61:I61"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8831,7 +10442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8996,23 +10607,17 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Konik Çatı Yapısal (CK1+CK2+KL1+diğer)</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>~5500</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>~5500</t>
-        </is>
+          <t>Konik Çatı Yapısal (CK1-CK4+KL1+W1+W2+YC1+YC2)</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>5454</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>5454</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
@@ -9344,23 +10949,17 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Merdiven + Korkuluk</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>Bekleniyor</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Bekleniyor</t>
-        </is>
+          <t>Merdiven + Korkuluk  (1 Komple)</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>1777</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>1777</v>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
@@ -9371,62 +10970,88 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>İSİM PLAK.</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Tank İsim Plakası (TI-1 ~ TI-4)</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>SAMANDIRA</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Mekanik Samandıra (N14)</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Bekleniyor</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Bekleniyor</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>MKD-206</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>BİLİNEN TOPLAM (yaklaşık, eksikler hariç):</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>~36898</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>~44134</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>~37346</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr"/>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>~44582</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:B23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add samandıra, bolt list, fix 351 plate error, add purchasing sheet
- Added Mekanik Samandıra (N14, 25 items, A283 Gr.C + SS A316L) to
  Manhol+Temizleme sheet based on MKD-206 drawing
- Added Çatım Civata-Somun-Rondela Listesi to Konik Çatı İskeleti:
  BOLT16×45 (CK3/CK4 bağlantısı, 4×48=192 adet) + BOLT20×50
  (YC1/YC2 bağlantısı, 4×24=96 adet), kl.8.8, DIN 7990/7989/4032
- Fixed maliyet sheet: "351 adet" → "31 adet" for 6mm govde plates,
  "~27 sektör" → "35 adet sektör" for tavan, updated Çatı weight to
  5454.0, Merdiven to 1777.0 in cost items
- Added new "Satınalma Metrajı" sheet (sheet 11) with:
  A) Plate steel by grade/thickness with piece counts and purchasing
     recommendations (S275J2 6/8/10/12/5mm net totals)
  B) Structural profiles and pipes summary
  C) Nozzle pipes and flanges (ASTM grades)
  D) Consolidated purchasing by steel class with 3% fire allowance

https://claude.ai/code/session_017Cpp1ZZqefHw5fPaaS3WRF
</commit_message>
<xml_diff>
--- a/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
+++ b/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Konik Çatı İskeleti" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Toplam Ağırlık Özeti" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Maliyet Tahmini" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Satınalma Metrajı" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -144,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -190,6 +191,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1064,16 +1071,23 @@
           <t>–</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>~5500</t>
-        </is>
+      <c r="E8" s="6" t="n">
+        <v>5454</v>
       </c>
       <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
+      <c r="G8" s="6">
+        <f>E8*F8</f>
+        <v/>
+      </c>
       <c r="H8" s="14" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr"/>
+      <c r="I8" s="6">
+        <f>E8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="6">
+        <f>G8+I8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1195,12 +1209,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>DİĞER</t>
+          <t>MERDİVEN</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Merdiven+Samandıra+Aksesuar</t>
+          <t>Merdiven + Korkuluk</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1213,16 +1227,23 @@
           <t>–</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>~500</t>
-        </is>
+      <c r="E12" s="6" t="n">
+        <v>1777</v>
       </c>
       <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
+      <c r="G12" s="6">
+        <f>E12*F12</f>
+        <v/>
+      </c>
       <c r="H12" s="14" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr"/>
+      <c r="I12" s="6">
+        <f>E12*H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="6">
+        <f>G12+I12</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1281,7 +1302,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>351 adet plaka</t>
+          <t>31 adet plaka</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1293,7 +1314,7 @@
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>1480×6000mm plakalar</t>
+          <t>POZ 3×30 + POZ 3A×1  |  1480×6000mm</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1343,7 @@
       <c r="F17" s="6" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>1480×6000mm + kısmi</t>
+          <t>POZ 1-1E×6 (6000mm) + POZ 2×1 (3997mm)</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1360,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>~27 adet sektör</t>
+          <t>35 adet sektör</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1351,7 +1372,7 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Konik şekil, özel kalıp</t>
+          <t>POZ 1-9 toplam 35 parça, 1500×6000mm stokundan</t>
         </is>
       </c>
     </row>
@@ -1824,6 +1845,1224 @@
     <mergeCell ref="A40:J40"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A33:J33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>7000 Bbl ÜRETİM TANKI  —  NET SATINALMA METRAJ ÖZETİ  (1 TANK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>A. SAC PLAKA — Kalınlık ve Malzeme Sınıfına Göre</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="35" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>KALINLIK
+(mm)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>KULLANIM YERİ</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>PARÇA
+ADETİ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>NET
+AĞIRLIK (kg)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>STANDART STOK ÖNERİSİ</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>NOTLAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Gövde Silindirik Kurslar (POZ 3, 3A)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>12964</v>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>32× 1500×6000×6mm (%2 fire)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>1480mm enine kesilecek; 30 adet tam + 1 adet kısmi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Gövde Alt Kurs (POZ 1,1A,1B,1C,1D,1E,2)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>3549.1</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>7× 1500×6000×8mm</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>6 adet 6000mm tam, 1 adet 3997mm kısmi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Tavan Konik Sektör Plakaları (POZ 1-9)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>8147</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>40× 1500×6000×8mm (%15 fire)</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Sektör şekil; 8mm+6mm gövde ile birleşik sipariş önerilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>8mm TOPLAM</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Gövde (7 pk) + Tavan (35 pk) birleşik</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>11696.1</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>~47 plaka 1500×6000×8mm</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>★ Sipariş miktarı</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Taban Orta Plakalar (POZ 1-8)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>8266.700000000001</v>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>12× 1500×6000×10mm</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Büyük plakalardan nested kesim — fire düşük</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Taban Annüler (Çevre) Plakalar (POZ 9, 9A)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>2854.4</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>4× 1500×6000×12mm</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>800mm en; 1500mm'lik plakadan boyuna bölünecek</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Taban Drenaj Strip Parçaları (POZ 10-13)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>50mm × çeşitli boy şerit</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Atık sacdan kesilebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>S275J2 TOPLAM SAC AĞIRLIĞI</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>35836.7</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>★ Ana sac siparişi toplam</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>B. YAPISAL PROFİL VE BORU</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>PROFİL / BORU</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>KULLANIM YERİ</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM ADET</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM BOY (mm)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM AĞIRLIK (kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>UNP240</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Çatı CK1+CK2 Rafterlar</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>136440</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>~3732</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>UNP200</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Çatı CK3 Purlin</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>29448</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>~744</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>UNP200</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Çatı CK4 Purlin</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>16248</v>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>~410</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>PIP 323.9×8 Boru</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Çatı KL1 Merkezi Kolon</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>9369</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>580.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>L60×5 Köşebent</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Çatı YC1+YC2</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>~46740</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>~417</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 8×200 (C200×8)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Merdiven Borda</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>çeşitli</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>~388</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>NPU100</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Merdiven Basamak</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>çeşitli</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>~288</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>L60×6 Köşebent</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Merdiven Korkuluk/Detay</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>~100+</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>çeşitli</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>~560</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>1 1/4" SCH Boru (Handrail)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Merdiven Korkuluk</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>70000</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>178.5</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>C. NOZUL BORULARI VE FLANŞLARI  (ASTM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME / TİP</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>STANDART</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>KULLANIM YERİ</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>ADET</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>AĞIRLIK (kg)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>NOTLAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>12" SCH XS Boru</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A106 Gr.B</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>N1+N4+N21</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>6 adet</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>~129</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>2×N1,2×N4 + N21×4</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8" SCH XS Boru</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A106 Gr.B</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>1 adet</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6" SCH XS Boru+Dirsek</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A106+A234WPB</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>N7A/B</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>2 komple set</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>~107.2</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Dirsek dahil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1" / 1.5" Boru</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A106 Gr.B</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>N9+N18</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>2 adet</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>12" 150# SO-RF Flanş</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A105</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>N1+N4+N21</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>6 adet</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>~174</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8" 150# SO-RF Flanş</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A105</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>1 adet</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6" 150# SO-RF Flanş</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A105</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>N7A/B</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>2 adet</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1" / 1.5" Flanş</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A105</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>N9+N18</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>2 adet</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>~5</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>D. KONSOLİDE AĞIRLIK — Çelik Sınıfına Göre Satınalma Özeti</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ÇELİK SINIFI</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>KULLANIM</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>NET AĞIRLIK (kg)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>FİRE PAYI (%3)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>SATINALMA (kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Ana Yapı Sacları (Gövde+Taban+Tavan)</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>35836.7</v>
+      </c>
+      <c r="D39" s="12" t="n">
+        <v>1075.1</v>
+      </c>
+      <c r="E39" s="12" t="n">
+        <v>36911.8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Yapısal (Çatı+Merdiven profil+plakalar)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>~7230</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>~220</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>~7450</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A106 Gr.B</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Nozul Boruları</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>~255</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>~260</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A105</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Nozul Flanşları</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>~205</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>~210</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>A193 Gr.B7 / A194 Gr.2H</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>Cıvata-Somun-Rondela</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Çizimden sipariş</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C + S.S. A316L</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Mekanik Samandıra</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>1 komple set</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>AISI C1030</t>
+        </is>
+      </c>
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>Ankraj (16 adet)</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>★ S275J2 sac siparişi: 6mm (~12964 kg) + 8mm (~11696 kg) + 10mm (~8267 kg) + 12mm (~2854 kg). Net toplam ~35781 kg. %3 fire ile ~36855 kg sipariş önerilir.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5861,7 +7100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8691,12 +9930,805 @@
       </c>
       <c r="G104" s="9" t="inlineStr"/>
     </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>MEKANİK SAMANDIRA (N14)  —  1 Adet  (A283 Gr.C + S.S. A316L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>POZ</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>ADET</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>AÇIKLAMA</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM
+AĞIRLIK(kg)</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM
+AĞIRLIK(kg)</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>NOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B108" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>ø21 BORU ......... 26</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B109" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>ø27 BORU ......... 130</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>S.S. A316L</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G109" s="6" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B110" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>ø400×6 PLAKA</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>S.S. A316L</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B111" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 300×6×1257 PLAKA</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>S.S. A316L</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G111" s="6" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B112" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 100×6×100 PLAKA</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>S.S. A316L</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G112" s="4" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 30×5×80 PLAKA</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G113" s="6" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 50×10×298 PLAKA</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 50×10×292 PLAKA</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G115" s="6" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 50×5×268 PLAKA</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B117" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 200×2×9000 PLAKA  (Seviye Göstergesi)</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E117" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G117" s="6" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 50×2×200 PLAKA</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B119" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>L 60×60×6×9514 PROFİL</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E119" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G119" s="6" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B120" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>[ 140×7×625 PROFİL</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B121" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C121" s="6" t="inlineStr">
+        <is>
+          <t>ø50 MAKARA</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E121" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G121" s="6" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B122" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 30×5×60 PLAKA</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B123" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 150×15×300 PLAKA</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E123" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G123" s="6" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B124" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>⊏ 30×3×60 PLAKA</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>ø5×20 mm KONİK VİDA / PUL</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G125" s="6" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B126" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>M8 SAPLAMA-SOMUN</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B127" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>M18 SAPLAMA-SOMUN</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E127" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G127" s="6" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B128" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>ø8 ÇELİK HALAT</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B129" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>ø12 ÇELİK HALAT</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E129" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G129" s="6" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B130" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>ø12 DEMİR</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>S.S. A316L</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B131" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>HALAT KLEMENSİ</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>S.S. A316L</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G131" s="6" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>L 60×60×6×195 PROFİL</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>A 283 Gr.C</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>NOT: Malzeme listesi 1 adet samandıra için verilmiştir. Ağırlık değerleri çizimde belirtilmemiştir.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A106:G106"/>
     <mergeCell ref="A104:E104"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A2:G2"/>
@@ -8704,6 +10736,7 @@
     <mergeCell ref="A64:G64"/>
     <mergeCell ref="A41:G41"/>
     <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A133:G133"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8715,7 +10748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10409,8 +12442,295 @@
         </is>
       </c>
     </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>ÇATIM CİVATA-SOMUN-RONDELA LİSTESİ  (Standart: DIN 7990 / 7989 / 4032)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="25" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>CİVATA TANIMI</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>ÇATIM-1</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>ÇATIM-2</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME
+SINIFI</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>ADET</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>STANDART</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>BOLT 16×45</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>CK3</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>CK1</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>BOLT 16×45</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>CK3</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>CK2</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>BOLT 16×45</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>CK4</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>CK1</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>BOLT 16×45</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>CK4</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>CK2</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>BOLT 20×50</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>YC1</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>CK1</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>BOLT 20×50</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>YC1</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>CK2</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>BOLT 20×50</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>YC2</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>CK1</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>BOLT 20×50</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>YC2</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>CK2</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>7990/7989/4032</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>TOPLAM: BOLT 16×45 → 192 adet  |  BOLT 20×50 → 96 adet  (her civata için 1 somun + 2 rondela)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="A25:I25"/>
     <mergeCell ref="A66:I66"/>
     <mergeCell ref="A56:I56"/>
@@ -10424,12 +12744,14 @@
     <mergeCell ref="A64:G64"/>
     <mergeCell ref="A59:G59"/>
     <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A68:I68"/>
     <mergeCell ref="A54:G54"/>
     <mergeCell ref="A30:I30"/>
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A61:I61"/>
+    <mergeCell ref="A78:I78"/>
     <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Maliyet Tahmini hatalar düzeltildi: Sump ayrıştırma, RF Pad etiketi, birim düzeltmeleri
- Taban: 11176.7+76.1 tek satırdan ayrıldı → Taban sacları 11176.7 + Drenaj Çukuru 76.1 ayrı kalem
- Annüler "dahil" satırı kaldırıldı (zaten 11176.7 içinde, çift sayım riski giderildi)
- Nozul satırı "RF Takviye Sacları dahil" olarak güncellendi (~140 kg fark açıklandı)
- "~37 ton" → 35913 kg (sayısal, doğru toplam)
- "~3000 kg" profil → 5454 kg (çizim toplam ağırlığı)
- Birim sütunundaki "ton" hataları "kg" olarak düzeltildi

https://claude.ai/code/session_017Cpp1ZZqefHw5fPaaS3WRF
</commit_message>
<xml_diff>
--- a/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
+++ b/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
@@ -948,7 +948,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Taban Plakaları (Orta)</t>
+          <t>Taban Plakaları (Orta 10mm + Annüler 12mm + Strip 5mm)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -958,11 +958,11 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5–12</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>11252.8</v>
+        <v>11176.7</v>
       </c>
       <c r="F5" s="14" t="inlineStr"/>
       <c r="G5" s="4">
@@ -987,7 +987,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Annüler Plakalar (Kenar)</t>
+          <t>Drenaj Çukuru (Sump) — Ayrı İmalat Kalemi</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -997,19 +997,26 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>dahil</t>
-        </is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>76.09999999999999</v>
       </c>
       <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
+      <c r="G6" s="6">
+        <f>E6*F6</f>
+        <v/>
+      </c>
       <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="I6" s="6">
+        <f>E6*H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="6">
+        <f>G6+I6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1097,12 +1104,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Tüm Nozullar (N1+N4+N7A/B+N8+N9+N18+N19+N21)</t>
+          <t>Tüm Nozullar + RF Takviye Sacları (N1+N4+N7A/B+N8+N9+N18+N19+N21)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>A106/A105</t>
+          <t>A106/A105/S275J2</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1302,7 +1309,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>31 adet plaka</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1331,7 +1338,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>7 adet plaka</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1360,7 +1367,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>35 adet sektör</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1384,24 +1391,22 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Tüm Plakalar</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>~37 ton</t>
-        </is>
+          <t>Tüm Ana Sac Plakalar (Gövde+Taban+Tavan+Sump)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>35913</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr"/>
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Gövde+Taban+Tavan</t>
+          <t>16513+11253+8147 = 35913 kg S275J2</t>
         </is>
       </c>
     </row>
@@ -1413,24 +1418,22 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>UNP240/UNP200/L80</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>~3000 kg</t>
-        </is>
+          <t>Yapısal Çelik Çatı İskeleti (UNP+PL+PIP+L)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>5454</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr"/>
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Çatı iskeleti</t>
+          <t>Çizim TOPLAM = 5454 kg S235JR</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1445,24 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>PIP 323.9×8 + Nozul boruları</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>~700 kg</t>
-        </is>
+          <t>PIP 323.9×8 + Nozul Boruları (A106 Gr.B)</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>700</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr"/>
       <c r="F21" s="6" t="inlineStr"/>
-      <c r="G21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Yaklaşık; kesin ağırlık nozul detay listesinden</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Sheet 11 yeniden yazıldı: Üretici/tedarikçi sipariş tablosu
- Eski karmaşık analiz tablosu kaldırıldı
- Yeni yapı: S.No | Tanım | Malzeme | Stok Boyut | Sipariş Adedi | Net Ağırlık | Birim Fiyat★ | Toplam
- Bölüm A: S275J2 sac (6mm/8mm/10mm/12mm) — 5 satır
- Bölüm B: S235JR profil/boru (UNP/PIP/L/NPU) — 9 satır
- Bölüm C: ASTM A106+A105 nozul boru/flanş — 9 satır
- Her bölüm alt toplamı + genel toplam formüllü
- Birim fiyat (G sütunu) sarı hücre, toplam formül =F*G

https://claude.ai/code/session_017Cpp1ZZqefHw5fPaaS3WRF
</commit_message>
<xml_diff>
--- a/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
+++ b/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,11 @@
       <b val="1"/>
       <color rgb="00FF0000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -192,11 +197,11 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1861,75 +1866,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>7000 Bbl ÜRETİM TANKI  —  NET SATINALMA METRAJ ÖZETİ  (1 TANK)</t>
+          <t>7000 Bbl ÜRETİM TANKI T-202  —  SATINALMA SİPARİŞ TABLOSU  (1 TANK)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>A. SAC PLAKA — Kalınlık ve Malzeme Sınıfına Göre</t>
+          <t>A — SAC PLAKA  (S275J2  |  EN 10025-3)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="35" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>S.NO</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>MALZEME</t>
+          <t>TANIM  /  MALZEME</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>KALINLIK
+          <t>MALZEME
+SINIFI</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>STOK BOYUT
 (mm)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>KULLANIM YERİ</t>
-        </is>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>PARÇA
-ADETİ</t>
+          <t>SİPARİŞ
+ADEDİ</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>NET
-AĞIRLIK (kg)</t>
+          <t>NET AĞIRLIK
+(kg)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>STANDART STOK ÖNERİSİ</t>
+          <t>BİRİM FİYAT ★
+($/kg)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>NOTLAR</t>
+          <t>TOPLAM
+($)</t>
         </is>
       </c>
     </row>
@@ -1937,331 +1945,296 @@
       <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Gövde Silindirik Sac — 2. ile 6. Kurs  (POZ 3, 3A)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>S275J2</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Gövde Silindirik Kurslar (POZ 3, 3A)</t>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>1500 × 6000 × 6</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F4" s="6" t="n">
         <v>12964</v>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>32× 1500×6000×6mm (%2 fire)</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>1480mm enine kesilecek; 30 adet tam + 1 adet kısmi</t>
-        </is>
+      <c r="G4" s="14" t="inlineStr"/>
+      <c r="H4" s="6">
+        <f>F4*G4</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Gövde Silindirik Sac — 1. Kurs (Alt)  (POZ 1, 1A–1E, 2)  +  Tavan Konik Sektör  (POZ 1–9)  [Birleşik Sipariş]</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>S275J2</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Gövde Alt Kurs (POZ 1,1A,1B,1C,1D,1E,2)</t>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1500 × 6000 × 8</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>3549.1</v>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>7× 1500×6000×8mm</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>6 adet 6000mm tam, 1 adet 3997mm kısmi</t>
-        </is>
+        <v>11696.1</v>
+      </c>
+      <c r="G5" s="14" t="inlineStr"/>
+      <c r="H5" s="4">
+        <f>F5*G5</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Taban Orta Plakalar  (POZ 1–8)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>S275J2</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Tavan Konik Sektör Plakaları (POZ 1-9)</t>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>1500 × 6000 × 10</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>8147</v>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>40× 1500×6000×8mm (%15 fire)</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Sektör şekil; 8mm+6mm gövde ile birleşik sipariş önerilir</t>
-        </is>
+        <v>8266.700000000001</v>
+      </c>
+      <c r="G6" s="14" t="inlineStr"/>
+      <c r="H6" s="6">
+        <f>F6*G6</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Taban Annüler (Çevre) Plakalar  (POZ 9, 9A)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>S275J2</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>8mm TOPLAM</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Gövde (7 pk) + Tavan (35 pk) birleşik</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>11696.1</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>~47 plaka 1500×6000×8mm</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>★ Sipariş miktarı</t>
-        </is>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1500 × 6000 × 12</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>2854.4</v>
+      </c>
+      <c r="G7" s="14" t="inlineStr"/>
+      <c r="H7" s="4">
+        <f>F7*G7</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Taban Drenaj Strip  (POZ 10–13)  — Atık sacdan kesilebilir</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>S275J2</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Taban Orta Plakalar (POZ 1-8)</t>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>50 geniş şerit</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>8266.700000000001</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>12× 1500×6000×10mm</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Büyük plakalardan nested kesim — fire düşük</t>
-        </is>
+        <v>55.5</v>
+      </c>
+      <c r="G8" s="14" t="inlineStr"/>
+      <c r="H8" s="6">
+        <f>F8*G8</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>A TOPLAM  —  S275J2 ANA SAC</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>35836.7</v>
+      </c>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="9">
+        <f>SUM(H4:H8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>B — YAPISAL PROFİL / BORU  (S235JR  |  EN 10025-2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="35" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>S.NO</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>TANIM  /  MALZEME</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME
+SINIFI</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>STOK BOYUT
+(mm)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>SİPARİŞ
+ADEDİ</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>NET AĞIRLIK
+(kg)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM FİYAT ★
+($/kg)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM
+($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>UNP 240 — Çatı Rafteri CK1 + CK2  (24 adet × 5685 mm)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>UNP240 × 12000</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>3732</v>
+      </c>
+      <c r="G13" s="14" t="inlineStr"/>
+      <c r="H13" s="4">
+        <f>F13*G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>UNP 200 — Çatı Purlin CK3  (24 adet × 1227 mm)</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>S235JR</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>UNP200 × 6000</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>S275J2</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Taban Annüler (Çevre) Plakalar (POZ 9, 9A)</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>2854.4</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>4× 1500×6000×12mm</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>800mm en; 1500mm'lik plakadan boyuna bölünecek</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>S275J2</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Taban Drenaj Strip Parçaları (POZ 10-13)</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>55.5</v>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>50mm × çeşitli boy şerit</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Atık sacdan kesilebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>S275J2</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>S275J2 TOPLAM SAC AĞIRLIĞI</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>35836.7</v>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>★ Ana sac siparişi toplam</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>B. YAPISAL PROFİL VE BORU</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>PROFİL / BORU</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>MALZEME</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>KULLANIM YERİ</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>TOPLAM ADET</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>TOPLAM BOY (mm)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>TOPLAM AĞIRLIK (kg)</t>
-        </is>
+      <c r="F14" s="6" t="n">
+        <v>744</v>
+      </c>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="6">
+        <f>F14*G14</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>UNP240</t>
+        <v>3</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>UNP 200 — Çatı Purlin CK4  (24 adet × 677 mm)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2271,28 +2244,28 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Çatı CK1+CK2 Rafterlar</t>
+          <t>UNP200 × 6000</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>136440</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>~3732</t>
-        </is>
+        <v>410.4</v>
+      </c>
+      <c r="G15" s="14" t="inlineStr"/>
+      <c r="H15" s="4">
+        <f>F15*G15</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>UNP200</t>
+        <v>4</v>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>PIP 323.9×8 — Çatı Merkezi Kolon KL1  (1 adet × 9369 mm)</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -2302,28 +2275,28 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Çatı CK3 Purlin</t>
+          <t>PIP323.9×8 × 12000</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>29448</v>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>~744</t>
-        </is>
+        <v>580.2</v>
+      </c>
+      <c r="G16" s="14" t="inlineStr"/>
+      <c r="H16" s="6">
+        <f>F16*G16</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>UNP200</t>
+        <v>5</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>L 60×5 Köşebent — Çatı YC1+YC2  (24 adet, toplam ~46740 mm)</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2333,28 +2306,28 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Çatı CK4 Purlin</t>
+          <t>L60×5 × 6000</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>16248</v>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>~410</t>
-        </is>
+        <v>417.6</v>
+      </c>
+      <c r="G17" s="14" t="inlineStr"/>
+      <c r="H17" s="4">
+        <f>F17*G17</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>PIP 323.9×8 Boru</t>
+        <v>6</v>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>C 200×8 (UPE200) — Merdiven Borda Kirişi  (8 adet, çeşitli boy)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -2364,26 +2337,28 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Çatı KL1 Merkezi Kolon</t>
+          <t>200×8 × 9000</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>9369</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>580.2</v>
+        <v>415.7</v>
+      </c>
+      <c r="G18" s="14" t="inlineStr"/>
+      <c r="H18" s="6">
+        <f>F18*G18</f>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>L60×5 Köşebent</t>
+        <v>7</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>NPU 100 — Merdiven Basamak  (13 adet × ~1080–1179 mm)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2393,30 +2368,28 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Çatı YC1+YC2</t>
+          <t>NPU100 × 6000</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>~46740</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>~417</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>288</v>
+      </c>
+      <c r="G19" s="14" t="inlineStr"/>
+      <c r="H19" s="4">
+        <f>F19*G19</f>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>⊏ 8×200 (C200×8)</t>
+        <v>8</v>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>L 60×6 Köşebent — Merdiven Korkuluk ve Detaylar  (~100+ parça)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2426,30 +2399,28 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Merdiven Borda</t>
+          <t>L60×6 × 6000</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>çeşitli</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>~388</t>
-        </is>
+        <v>20</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>499.6</v>
+      </c>
+      <c r="G20" s="14" t="inlineStr"/>
+      <c r="H20" s="6">
+        <f>F20*G20</f>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>NPU100</t>
+        <v>9</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>1¼" STD SCH Boru — Merdiven Korkuluk (Handrail)  (70000 mm)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2459,138 +2430,129 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Merdiven Basamak</t>
+          <t>1¼" SCH × 6000</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>çeşitli</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>~288</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="G21" s="14" t="inlineStr"/>
+      <c r="H21" s="4">
+        <f>F21*G21</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>L60×6 Köşebent</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Merdiven Korkuluk/Detay</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>~100+</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>çeşitli</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>~560</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>1 1/4" SCH Boru (Handrail)</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Merdiven Korkuluk</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>70000</v>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>178.5</v>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>C. NOZUL BORULARI VE FLANŞLARI  (ASTM)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>MALZEME / TİP</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>STANDART</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>KULLANIM YERİ</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>ADET</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>AĞIRLIK (kg)</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>NOTLAR</t>
-        </is>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>B TOPLAM  —  S235JR YAPISAL</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>7266</v>
+      </c>
+      <c r="G22" s="9" t="inlineStr"/>
+      <c r="H22" s="9">
+        <f>SUM(H13:H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>C — NOZUL BORU / FLANŞ  (ASTM A106 Gr.B  +  ASTM A105)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>S.NO</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>TANIM  /  MALZEME</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>MALZEME
+SINIFI</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>STOK BOYUT
+(mm)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>SİPARİŞ
+ADEDİ</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>NET AĞIRLIK
+(kg)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>BİRİM FİYAT ★
+($/kg)</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>TOPLAM
+($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>12" SCH XS Boru — N1 Giriş + N4 Çıkış + N21 Hava (6 adet × ~223–290 mm)</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>ASTM A106 Gr.B</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>12" SCH XS × 6000</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>129</v>
+      </c>
+      <c r="G26" s="14" t="inlineStr"/>
+      <c r="H26" s="6">
+        <f>F26*G26</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>12" SCH XS Boru</t>
+        <v>2</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>8" SCH XS Boru — N8 Köpük Yapıcı  (1 adet × 221 mm)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2600,32 +2562,28 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>N1+N4+N21</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>6 adet</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>~129</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>2×N1,2×N4 + N21×4</t>
-        </is>
+          <t>8" SCH XS × 6000</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G27" s="14" t="inlineStr"/>
+      <c r="H27" s="4">
+        <f>F27*G27</f>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 8" SCH XS Boru</t>
+        <v>3</v>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>6" SCH XS Boru — N7A/B Drain  (2 set: 360+870+540 mm + 90° Dirsek)</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -2635,63 +2593,59 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>N8</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>1 adet</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr"/>
+          <t>6" SCH XS × 6000</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="G28" s="14" t="inlineStr"/>
+      <c r="H28" s="6">
+        <f>F28*G28</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6" SCH XS Boru+Dirsek</t>
+        <v>4</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>6" SCH XS 90° LR Dirsek — N7A/B Drain  (2 adet)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>ASTM A106+A234WPB</t>
+          <t>ASTM A234 WPB</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>N7A/B</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>2 komple set</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>~107.2</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Dirsek dahil</t>
-        </is>
+          <t>6" SCH XS Elbow</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G29" s="14" t="inlineStr"/>
+      <c r="H29" s="4">
+        <f>F29*G29</f>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 1" / 1.5" Boru</t>
+        <v>5</v>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>1½" SCH XS Boru — N9 Sıcaklık  +  1" SCH XS Boru — N18 Seviye</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2701,28 +2655,28 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>N9+N18</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>2 adet</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>~8</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr"/>
+          <t>1½"+1" SCH XS × 1000</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G30" s="14" t="inlineStr"/>
+      <c r="H30" s="6">
+        <f>F30*G30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>12" 150# SO-RF Flanş</t>
+        <v>6</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>12" 150# SO-RF Flanş — N1 + N4 + N21  (6 adet)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2732,28 +2686,28 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>N1+N4+N21</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>6 adet</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>~174</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr"/>
+          <t>12" 150# SO-RF</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="G31" s="14" t="inlineStr"/>
+      <c r="H31" s="4">
+        <f>F31*G31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 8" 150# SO-RF Flanş</t>
+        <v>7</v>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>8" 150# SO-RF Flanş — N8  (1 adet)</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2763,26 +2717,28 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>N8</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>1 adet</t>
-        </is>
+          <t>8" 150# SO-RF</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="F32" s="6" t="n">
         <v>13.5</v>
       </c>
-      <c r="G32" s="6" t="inlineStr"/>
+      <c r="G32" s="14" t="inlineStr"/>
+      <c r="H32" s="6">
+        <f>F32*G32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 6" 150# SO-RF Flanş</t>
+        <v>8</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>6" 150# SO-RF Flanş — N7A/B  (2 adet)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2792,26 +2748,28 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>N7A/B</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>2 adet</t>
-        </is>
+          <t>6" 150# SO-RF</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>11.8</v>
       </c>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="G33" s="14" t="inlineStr"/>
+      <c r="H33" s="4">
+        <f>F33*G33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 1" / 1.5" Flanş</t>
+        <v>9</v>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>1½" 150# SO-RF Flanş — N9  +  1" 150# SO-RF Flanş — N18  (2 adet)</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2821,253 +2779,69 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>N9+N18</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>2 adet</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>~5</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>D. KONSOLİDE AĞIRLIK — Çelik Sınıfına Göre Satınalma Özeti</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>ÇELİK SINIFI</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>KULLANIM</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>NET AĞIRLIK (kg)</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>FİRE PAYI (%3)</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>SATINALMA (kg)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>S275J2</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>Ana Yapı Sacları (Gövde+Taban+Tavan)</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="n">
-        <v>35836.7</v>
-      </c>
-      <c r="D39" s="12" t="n">
-        <v>1075.1</v>
-      </c>
-      <c r="E39" s="12" t="n">
-        <v>36911.8</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>Yapısal (Çatı+Merdiven profil+plakalar)</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>~7230</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>~220</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>~7450</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>ASTM A106 Gr.B</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>Nozul Boruları</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>~255</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>~260</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>ASTM A105</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="inlineStr">
-        <is>
-          <t>Nozul Flanşları</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>~205</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>~210</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>A193 Gr.B7 / A194 Gr.2H</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>Cıvata-Somun-Rondela</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>Çizimden sipariş</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>A 283 Gr.C + S.S. A316L</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>Mekanik Samandıra</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>1 komple set</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>AISI C1030</t>
-        </is>
-      </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>Ankraj (16 adet)</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>216</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>220</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t>★ S275J2 sac siparişi: 6mm (~12964 kg) + 8mm (~11696 kg) + 10mm (~8267 kg) + 12mm (~2854 kg). Net toplam ~35781 kg. %3 fire ile ~36855 kg sipariş önerilir.</t>
+          <t>1½"+1" 150# SO-RF</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="G34" s="14" t="inlineStr"/>
+      <c r="H34" s="6">
+        <f>F34*G34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>C TOPLAM  —  ASTM BORU + FLANŞ</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>402.1</v>
+      </c>
+      <c r="G35" s="9" t="inlineStr"/>
+      <c r="H35" s="9">
+        <f>SUM(H26:H34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>GENEL TOPLAM  (A + B + C)  —  Birim Fiyatlar Girildiğinde Otomatik Hesaplanır</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="n">
+        <v>43504.8</v>
+      </c>
+      <c r="G37" s="1" t="inlineStr"/>
+      <c r="H37" s="1">
+        <f>H10+H23+H36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>★ G sütununa (BİRİM FİYAT) $/kg değeri giriniz. Bölüm D malzemeleri (Cıvata/Somun/Rondela, Samandıra, Ankraj) ayrıca fiyatlandırılacaktır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A25:H25"/>
+  <mergeCells count="9">
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sheet 11 profil bölümü düzeltildi: bar adedi hataları ve kafa karıştıran yapı
- C200×8 borda: 9 bar → 4 bar (nesting hesabı ile: 4×9000mm)
- NPU100 basamak: 3 bar → 5 bar (24 parça/27102mm doğru)
- UNP200 CK3+CK4 ayrı satır (7 bar) → tek satır 8 bar (birlikte sipariş)
- Her satır tanımına "→ X parça × Ymm | Z bar sipariş" mantığı eklendi
- Sipariş adedi neden o sayı olduğu görünür hale getirildi

https://claude.ai/code/session_017Cpp1ZZqefHw5fPaaS3WRF
</commit_message>
<xml_diff>
--- a/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
+++ b/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -196,6 +196,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1866,7 +1869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2166,13 +2169,14 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>UNP 240 — Çatı Rafteri CK1 + CK2  (24 adet × 5685 mm)</t>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>UNP 240  —  Çatı Rafteri CK1+CK2
+→ 24 parça × 5685 mm  |  12000mm bar'dan 2 parça  |  12 bar sipariş</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -2197,13 +2201,14 @@
         <v/>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>UNP 200 — Çatı Purlin CK3  (24 adet × 1227 mm)</t>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>UNP 200  —  Çatı Purlin CK3 + CK4
+→ CK3: 24×1227mm + CK4: 24×677mm = 45696mm  |  8 bar sipariş</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -2217,10 +2222,10 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>744</v>
+        <v>1154.4</v>
       </c>
       <c r="G14" s="14" t="inlineStr"/>
       <c r="H14" s="6">
@@ -2228,13 +2233,14 @@
         <v/>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>UNP 200 — Çatı Purlin CK4  (24 adet × 677 mm)</t>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>PIP 323.9×8  —  Çatı Merkezi Kolon KL1
+→ 1 parça × 9369 mm  |  1 bar 12000mm sipariş</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2244,14 +2250,14 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>UNP200 × 6000</t>
+          <t>PIP 323.9×8 × 12000</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>410.4</v>
+        <v>580.2</v>
       </c>
       <c r="G15" s="14" t="inlineStr"/>
       <c r="H15" s="4">
@@ -2259,13 +2265,14 @@
         <v/>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>PIP 323.9×8 — Çatı Merkezi Kolon KL1  (1 adet × 9369 mm)</t>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>L 60×5  —  Çatı Yatay Çelik YC1+YC2
+→ YC1: 12×1931mm + YC2: 12×1954mm = 46620mm  |  8 bar sipariş</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -2275,14 +2282,14 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>PIP323.9×8 × 12000</t>
+          <t>L60×5 × 6000</t>
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>580.2</v>
+        <v>417.6</v>
       </c>
       <c r="G16" s="14" t="inlineStr"/>
       <c r="H16" s="6">
@@ -2290,13 +2297,14 @@
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>L 60×5 Köşebent — Çatı YC1+YC2  (24 adet, toplam ~46740 mm)</t>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>C 200×8  —  Merdiven Borda Kirişi
+→ 9 parça / 33096mm toplam  |  9000mm bar'a nesting: 4 bar sipariş</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2306,14 +2314,14 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>L60×5 × 6000</t>
+          <t>200×8 × 9000</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>417.6</v>
+        <v>415.7</v>
       </c>
       <c r="G17" s="14" t="inlineStr"/>
       <c r="H17" s="4">
@@ -2321,13 +2329,14 @@
         <v/>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>C 200×8 (UPE200) — Merdiven Borda Kirişi  (8 adet, çeşitli boy)</t>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>NPU 100  —  Merdiven Basamak
+→ 12×1080mm + 12×1179mm = 27102mm  |  5 bar sipariş</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -2337,14 +2346,14 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>200×8 × 9000</t>
+          <t>NPU100 × 6000</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>415.7</v>
+        <v>288</v>
       </c>
       <c r="G18" s="14" t="inlineStr"/>
       <c r="H18" s="6">
@@ -2352,13 +2361,14 @@
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>NPU 100 — Merdiven Basamak  (13 adet × ~1080–1179 mm)</t>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>L 60×6  —  Merdiven Korkuluk ve Bağlantı Detayları
+→ ~100+ parça / ~87000mm toplam  |  15 bar sipariş</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2368,14 +2378,14 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>NPU100 × 6000</t>
+          <t>L60×6 × 6000</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>288</v>
+        <v>499.6</v>
       </c>
       <c r="G19" s="14" t="inlineStr"/>
       <c r="H19" s="4">
@@ -2383,13 +2393,14 @@
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>L 60×6 Köşebent — Merdiven Korkuluk ve Detaylar  (~100+ parça)</t>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>1¼" STD SCH Pipe  —  Merdiven Küpeşte (Handrail)
+→ 1 bütün parça 70000mm  |  12 boy 6000mm sipariş</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2399,14 +2410,14 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>L60×6 × 6000</t>
+          <t>1¼" SCH × 6000</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>499.6</v>
+        <v>178.5</v>
       </c>
       <c r="G20" s="14" t="inlineStr"/>
       <c r="H20" s="6">
@@ -2415,113 +2426,113 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>1¼" STD SCH Boru — Merdiven Korkuluk (Handrail)  (70000 mm)</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>S235JR</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>1¼" SCH × 6000</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>178.5</v>
-      </c>
-      <c r="G21" s="14" t="inlineStr"/>
-      <c r="H21" s="4">
-        <f>F21*G21</f>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>B TOPLAM  —  S235JR YAPISAL</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>7266</v>
+      </c>
+      <c r="G21" s="9" t="inlineStr"/>
+      <c r="H21" s="9">
+        <f>SUM(H13:H20)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>B TOPLAM  —  S235JR YAPISAL</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>7266</v>
-      </c>
-      <c r="G22" s="9" t="inlineStr"/>
-      <c r="H22" s="9">
-        <f>SUM(H13:H21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>C — NOZUL BORU / FLANŞ  (ASTM A106 Gr.B  +  ASTM A105)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="35" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>S.NO</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>TANIM  /  MALZEME</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>MALZEME
 SINIFI</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>STOK BOYUT
 (mm)</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>SİPARİŞ
 ADEDİ</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>NET AĞIRLIK
 (kg)</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>BİRİM FİYAT ★
 ($/kg)</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>TOPLAM
 ($)</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>12" SCH XS Boru — N1 Giriş + N4 Çıkış + N21 Hava (6 adet × ~223–290 mm)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>ASTM A106 Gr.B</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>12" SCH XS × 6000</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="G25" s="14" t="inlineStr"/>
+      <c r="H25" s="4">
+        <f>F25*G25</f>
+        <v/>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>12" SCH XS Boru — N1 Giriş + N4 Çıkış + N21 Hava (6 adet × ~223–290 mm)</t>
+          <t>8" SCH XS Boru — N8 Köpük Yapıcı  (1 adet × 221 mm)</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -2531,14 +2542,14 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>12" SCH XS × 6000</t>
+          <t>8" SCH XS × 6000</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>129</v>
+        <v>11.4</v>
       </c>
       <c r="G26" s="14" t="inlineStr"/>
       <c r="H26" s="6">
@@ -2548,11 +2559,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>8" SCH XS Boru — N8 Köpük Yapıcı  (1 adet × 221 mm)</t>
+          <t>6" SCH XS Boru — N7A/B Drain  (2 set: 360+870+540 mm + 90° Dirsek)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2562,14 +2573,14 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>8" SCH XS × 6000</t>
+          <t>6" SCH XS × 6000</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>11.4</v>
+        <v>47.2</v>
       </c>
       <c r="G27" s="14" t="inlineStr"/>
       <c r="H27" s="4">
@@ -2579,28 +2590,28 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>6" SCH XS Boru — N7A/B Drain  (2 set: 360+870+540 mm + 90° Dirsek)</t>
+          <t>6" SCH XS 90° LR Dirsek — N7A/B Drain  (2 adet)</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>ASTM A106 Gr.B</t>
+          <t>ASTM A234 WPB</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>6" SCH XS × 6000</t>
+          <t>6" SCH XS Elbow</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>47.2</v>
+        <v>10.8</v>
       </c>
       <c r="G28" s="14" t="inlineStr"/>
       <c r="H28" s="6">
@@ -2610,28 +2621,28 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>6" SCH XS 90° LR Dirsek — N7A/B Drain  (2 adet)</t>
+          <t>1½" SCH XS Boru — N9 Sıcaklık  +  1" SCH XS Boru — N18 Seviye</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>ASTM A234 WPB</t>
+          <t>ASTM A106 Gr.B</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>6" SCH XS Elbow</t>
+          <t>1½"+1" SCH XS × 1000</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>10.8</v>
+        <v>1.4</v>
       </c>
       <c r="G29" s="14" t="inlineStr"/>
       <c r="H29" s="4">
@@ -2641,28 +2652,28 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>1½" SCH XS Boru — N9 Sıcaklık  +  1" SCH XS Boru — N18 Seviye</t>
+          <t>12" 150# SO-RF Flanş — N1 + N4 + N21  (6 adet)</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>ASTM A106 Gr.B</t>
+          <t>ASTM A105</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>1½"+1" SCH XS × 1000</t>
+          <t>12" 150# SO-RF</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>1.4</v>
+        <v>174</v>
       </c>
       <c r="G30" s="14" t="inlineStr"/>
       <c r="H30" s="6">
@@ -2672,11 +2683,11 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>12" 150# SO-RF Flanş — N1 + N4 + N21  (6 adet)</t>
+          <t>8" 150# SO-RF Flanş — N8  (1 adet)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2686,14 +2697,14 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>12" 150# SO-RF</t>
+          <t>8" 150# SO-RF</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>174</v>
+        <v>13.5</v>
       </c>
       <c r="G31" s="14" t="inlineStr"/>
       <c r="H31" s="4">
@@ -2703,11 +2714,11 @@
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>8" 150# SO-RF Flanş — N8  (1 adet)</t>
+          <t>6" 150# SO-RF Flanş — N7A/B  (2 adet)</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2717,14 +2728,14 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>8" 150# SO-RF</t>
+          <t>6" 150# SO-RF</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>13.5</v>
+        <v>11.8</v>
       </c>
       <c r="G32" s="14" t="inlineStr"/>
       <c r="H32" s="6">
@@ -2734,11 +2745,11 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>6" 150# SO-RF Flanş — N7A/B  (2 adet)</t>
+          <t>1½" 150# SO-RF Flanş — N9  +  1" 150# SO-RF Flanş — N18  (2 adet)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2748,14 +2759,14 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>6" 150# SO-RF</t>
+          <t>1½"+1" 150# SO-RF</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>11.8</v>
+        <v>2.95</v>
       </c>
       <c r="G33" s="14" t="inlineStr"/>
       <c r="H33" s="4">
@@ -2764,68 +2775,37 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>1½" 150# SO-RF Flanş — N9  +  1" 150# SO-RF Flanş — N18  (2 adet)</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>ASTM A105</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>1½"+1" 150# SO-RF</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" s="6" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="G34" s="14" t="inlineStr"/>
-      <c r="H34" s="6">
-        <f>F34*G34</f>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>C TOPLAM  —  ASTM BORU + FLANŞ</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>402.1</v>
+      </c>
+      <c r="G34" s="9" t="inlineStr"/>
+      <c r="H34" s="9">
+        <f>SUM(H25:H33)</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>C TOPLAM  —  ASTM BORU + FLANŞ</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n">
-        <v>402.1</v>
-      </c>
-      <c r="G35" s="9" t="inlineStr"/>
-      <c r="H35" s="9">
-        <f>SUM(H26:H34)</f>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>GENEL TOPLAM  (A + B + C)  —  Birim Fiyatlar Girildiğinde Otomatik Hesaplanır</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="n">
+        <v>43504.8</v>
+      </c>
+      <c r="G36" s="1" t="inlineStr"/>
+      <c r="H36" s="1">
+        <f>H10+H22+H35</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>GENEL TOPLAM  (A + B + C)  —  Birim Fiyatlar Girildiğinde Otomatik Hesaplanır</t>
-        </is>
-      </c>
-      <c r="F37" s="1" t="n">
-        <v>43504.8</v>
-      </c>
-      <c r="G37" s="1" t="inlineStr"/>
-      <c r="H37" s="1">
-        <f>H10+H23+H36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>★ G sütununa (BİRİM FİYAT) $/kg değeri giriniz. Bölüm D malzemeleri (Cıvata/Somun/Rondela, Samandıra, Ankraj) ayrıca fiyatlandırılacaktır.</t>
         </is>
@@ -2833,14 +2813,14 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A36:E36"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
T-202 gövde düzeltme: POZ 3=29 adet, POZ 3B eklendi
- POZ 3: 30→29 adet, toplam 12546.0→12127.8 kg (çizim hatası düzeltildi)
- POZ 3B: 1 adet, 1480×6×6000, 418.0 kg (eksik satır eklendi)
- Kurs özeti: "POZ 3×29 + POZ 3A×1 + POZ 3B×1 = 31 adet"
- Her iki Excel dosyası yeniden üretildi
</commit_message>
<xml_diff>
--- a/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
+++ b/7000Bbl_Tank_Malzeme_ve_Maliyet.xlsx
@@ -3984,7 +3984,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
         <v>418.2</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>12546</v>
+        <v>12127.8</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>6</v>
@@ -4045,17 +4045,51 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>⊏ 1480×6 ......... 6000</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>S275J2</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Kesim + Silindirik Bükme</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>TOPLAM AĞIRLIK:</t>
         </is>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F13" s="9" t="n">
         <v>16513</v>
       </c>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
+      <c r="G13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -4150,7 +4184,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>31 adet (POZ 3×30 + POZ 3A×1)</t>
+          <t>31 adet (POZ 3×29 + POZ 3A×1 + POZ 3B×1)</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -4164,21 +4198,21 @@
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>12964</v>
+        <v>12963.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>NOT: Kurs yüksekliği 1480mm, toplam gövde yüksekliği ≈ 6 × 1480mm = 8880mm ≈ 8.920m. POZ 3 = 30 adet standart silindirik plaka (8mm'lik kursun nozulsuz plakaları 8mm'dir).</t>
+          <t>NOT: Kurs yüksekliği 1480mm, toplam gövde yüksekliği ≈ 6 × 1480mm = 8880mm ≈ 8.920m. POZ 3 = 29 adet standart, POZ 3A ve 3B = kapama plakaları (toplam 31 adet 6mm). Çizimdeki '12546' toplam değeri drawing hatasıdır; doğrusu 12127.8 kg (29×418.2).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>